<commit_message>
Moving all census data processing to census_data_process
</commit_message>
<xml_diff>
--- a/Data/unitary_authority_data.xlsx
+++ b/Data/unitary_authority_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scotsconnect-my.sharepoint.com/personal/euan_wakefield_gov_scot/Documents/R/RESAS-Agricultural-Statistics-Hub/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://scotsconnect-my.sharepoint.com/personal/calli_dougall_gov_scot/Documents/RESAS/RESAS-Agricultural-Statistics-Hub2/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="2" documentId="8_{804F3F20-43A3-4563-8B5B-8A0BE0CF2310}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C9586194-A63C-4EF9-893B-07B08E8CABE4}"/>
   <bookViews>
-    <workbookView xWindow="17" yWindow="17" windowWidth="16440" windowHeight="8520" firstSheet="1" activeTab="1" xr2:uid="{B086D461-E5E0-4CA5-AF09-B2445CFA5063}"/>
+    <workbookView minimized="1" xWindow="2110" yWindow="1460" windowWidth="14400" windowHeight="7280" xr2:uid="{B086D461-E5E0-4CA5-AF09-B2445CFA5063}"/>
   </bookViews>
   <sheets>
     <sheet name="unitary_crops_area" sheetId="1" r:id="rId1"/>
@@ -887,18 +887,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{517F41B0-8BE9-4AEE-A1F7-25416572F43D}">
   <dimension ref="A1:Z34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.23046875" style="3"/>
-    <col min="2" max="20" width="9.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="23" width="10.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="10.69140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.3828125" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="16384" width="9.23046875" style="3"/>
+    <col min="1" max="1" width="9.26953125" style="3"/>
+    <col min="2" max="20" width="9.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="21" max="23" width="10.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.36328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="27" max="16384" width="9.26953125" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="46.3" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" ht="46.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -978,7 +978,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>26</v>
       </c>
@@ -1058,7 +1058,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>27</v>
       </c>
@@ -1218,7 +1218,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>29</v>
       </c>
@@ -1298,7 +1298,7 @@
         <v>1846</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>30</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>31</v>
       </c>
@@ -1458,7 +1458,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="60" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" ht="62" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>3950</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>33</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>34</v>
       </c>
@@ -1698,7 +1698,7 @@
         <v>1155</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>35</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>36</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>550</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>1444</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>40</v>
       </c>
@@ -2178,7 +2178,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>41</v>
       </c>
@@ -2258,7 +2258,7 @@
         <v>9161</v>
       </c>
     </row>
-    <row r="18" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>42</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="19" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>43</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="21" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>45</v>
       </c>
@@ -2578,7 +2578,7 @@
         <v>5237</v>
       </c>
     </row>
-    <row r="22" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>46</v>
       </c>
@@ -2658,7 +2658,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="23" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>47</v>
       </c>
@@ -2738,7 +2738,7 @@
         <v>486</v>
       </c>
     </row>
-    <row r="24" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>48</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>1736</v>
       </c>
     </row>
-    <row r="25" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>49</v>
       </c>
@@ -2898,7 +2898,7 @@
         <v>2330</v>
       </c>
     </row>
-    <row r="26" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>50</v>
       </c>
@@ -2978,7 +2978,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="27" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>51</v>
       </c>
@@ -3058,7 +3058,7 @@
         <v>2543</v>
       </c>
     </row>
-    <row r="28" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>52</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>1706</v>
       </c>
     </row>
-    <row r="29" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>53</v>
       </c>
@@ -3218,7 +3218,7 @@
         <v>891</v>
       </c>
     </row>
-    <row r="30" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>54</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>905</v>
       </c>
     </row>
-    <row r="32" spans="1:26" ht="45" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:26" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>56</v>
       </c>
@@ -3458,7 +3458,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>57</v>
       </c>
@@ -3538,7 +3538,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="34" spans="1:26" ht="30" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:26" ht="31" x14ac:dyDescent="0.35">
       <c r="A34" s="9" t="s">
         <v>58</v>
       </c>
@@ -3626,28 +3626,28 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BE4FAE2-FEDB-4032-AB05-A5EBE0B80136}">
   <dimension ref="A1:AJ33"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="4" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.765625" bestFit="1" customWidth="1"/>
-    <col min="6" max="15" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="9.765625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.23046875" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="10.23046875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.3828125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="9.765625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.3828125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="9.765625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="11.3828125" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="31" max="36" width="9.3828125" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="15" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="36" width="9.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" ht="135.44999999999999" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:36" ht="170.5" x14ac:dyDescent="0.35">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -3757,7 +3757,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>26</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>27</v>
       </c>
@@ -3977,7 +3977,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="4" spans="1:36" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>28</v>
       </c>
@@ -4087,7 +4087,7 @@
         <v>340</v>
       </c>
     </row>
-    <row r="5" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>29</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>30</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>31</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:36" ht="60.45" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:36" ht="62" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="9" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>33</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>34</v>
       </c>
@@ -4747,7 +4747,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:36" ht="62" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>35</v>
       </c>
@@ -4857,7 +4857,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="12" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>36</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="13" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -5077,7 +5077,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="14" spans="1:36" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>38</v>
       </c>
@@ -5187,7 +5187,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="15" spans="1:36" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>39</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>40</v>
       </c>
@@ -5407,7 +5407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>41</v>
       </c>
@@ -5517,7 +5517,7 @@
         <v>952</v>
       </c>
     </row>
-    <row r="18" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>42</v>
       </c>
@@ -5627,7 +5627,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>43</v>
       </c>
@@ -5737,7 +5737,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="20" spans="1:36" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>44</v>
       </c>
@@ -5847,7 +5847,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="21" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>45</v>
       </c>
@@ -5957,7 +5957,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>46</v>
       </c>
@@ -6067,7 +6067,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="23" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>47</v>
       </c>
@@ -6177,7 +6177,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="24" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>48</v>
       </c>
@@ -6287,7 +6287,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="25" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>49</v>
       </c>
@@ -6397,7 +6397,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="26" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>50</v>
       </c>
@@ -6507,7 +6507,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="27" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>51</v>
       </c>
@@ -6617,7 +6617,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="28" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>52</v>
       </c>
@@ -6727,7 +6727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>53</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:36" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>54</v>
       </c>
@@ -6947,7 +6947,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="31" spans="1:36" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:36" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>55</v>
       </c>
@@ -7057,7 +7057,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="32" spans="1:36" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:36" ht="62" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>56</v>
       </c>
@@ -7167,7 +7167,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:36" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:36" ht="31" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>57</v>
       </c>
@@ -7285,9 +7285,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E865701F-7324-46CB-BFA5-E1B1525C72CE}">
   <dimension ref="A1:Y33"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:25" ht="138.9" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:25" ht="139.5" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -7364,7 +7364,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>26</v>
       </c>
@@ -7441,7 +7441,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="3" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>27</v>
       </c>
@@ -7518,7 +7518,7 @@
         <v>8775</v>
       </c>
     </row>
-    <row r="4" spans="1:25" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:25" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>28</v>
       </c>
@@ -7595,7 +7595,7 @@
         <v>3992</v>
       </c>
     </row>
-    <row r="5" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>29</v>
       </c>
@@ -7672,7 +7672,7 @@
         <v>2614</v>
       </c>
     </row>
-    <row r="6" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>30</v>
       </c>
@@ -7749,7 +7749,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="7" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A7" s="4" t="s">
         <v>31</v>
       </c>
@@ -7826,7 +7826,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="8" spans="1:25" ht="60.45" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:25" ht="62" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>32</v>
       </c>
@@ -7903,7 +7903,7 @@
         <v>7096</v>
       </c>
     </row>
-    <row r="9" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>33</v>
       </c>
@@ -7980,7 +7980,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="10" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>34</v>
       </c>
@@ -8057,7 +8057,7 @@
         <v>1863</v>
       </c>
     </row>
-    <row r="11" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:25" ht="62" x14ac:dyDescent="0.35">
       <c r="A11" s="4" t="s">
         <v>35</v>
       </c>
@@ -8134,7 +8134,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>36</v>
       </c>
@@ -8211,7 +8211,7 @@
         <v>1497</v>
       </c>
     </row>
-    <row r="13" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>37</v>
       </c>
@@ -8288,7 +8288,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="14" spans="1:25" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:25" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>38</v>
       </c>
@@ -8365,7 +8365,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="15" spans="1:25" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:25" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>39</v>
       </c>
@@ -8442,7 +8442,7 @@
         <v>3387</v>
       </c>
     </row>
-    <row r="16" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>40</v>
       </c>
@@ -8519,7 +8519,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="17" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>41</v>
       </c>
@@ -8596,7 +8596,7 @@
         <v>9822</v>
       </c>
     </row>
-    <row r="18" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>42</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>43</v>
       </c>
@@ -8750,7 +8750,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="20" spans="1:25" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:25" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="4" t="s">
         <v>44</v>
       </c>
@@ -8827,7 +8827,7 @@
         <v>1768</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>45</v>
       </c>
@@ -8904,7 +8904,7 @@
         <v>3587</v>
       </c>
     </row>
-    <row r="22" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>46</v>
       </c>
@@ -8981,7 +8981,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="23" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>47</v>
       </c>
@@ -9058,7 +9058,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="24" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A24" s="4" t="s">
         <v>48</v>
       </c>
@@ -9135,7 +9135,7 @@
         <v>1905</v>
       </c>
     </row>
-    <row r="25" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>49</v>
       </c>
@@ -9212,7 +9212,7 @@
         <v>4522</v>
       </c>
     </row>
-    <row r="26" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>50</v>
       </c>
@@ -9289,7 +9289,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="27" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>51</v>
       </c>
@@ -9366,7 +9366,7 @@
         <v>4253</v>
       </c>
     </row>
-    <row r="28" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>52</v>
       </c>
@@ -9443,7 +9443,7 @@
         <v>1843</v>
       </c>
     </row>
-    <row r="29" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>53</v>
       </c>
@@ -9520,7 +9520,7 @@
         <v>1340</v>
       </c>
     </row>
-    <row r="30" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:25" ht="46.5" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>54</v>
       </c>
@@ -9597,7 +9597,7 @@
         <v>2176</v>
       </c>
     </row>
-    <row r="31" spans="1:25" ht="15.45" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:25" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="4" t="s">
         <v>55</v>
       </c>
@@ -9674,7 +9674,7 @@
         <v>1204</v>
       </c>
     </row>
-    <row r="32" spans="1:25" ht="45.45" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:25" ht="62" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>56</v>
       </c>
@@ -9751,7 +9751,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="33" spans="1:25" ht="30.45" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:25" ht="31" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>57</v>
       </c>

</xml_diff>